<commit_message>
Updated to enable animal shapekeys
</commit_message>
<xml_diff>
--- a/src/assets/Sources.xlsx
+++ b/src/assets/Sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camer\OneDrive\Documents\GitHub\Madhatters-Table-Top-RPG-Mini-Maker\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D774B731-37E8-4541-A018-63865503852F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06550DB9-2256-4477-8056-054E5B9F8D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6690" yWindow="3360" windowWidth="21600" windowHeight="11505" xr2:uid="{61C89FE4-8FBE-4549-A785-404B3EAD14AE}"/>
+    <workbookView xWindow="4380" yWindow="1935" windowWidth="21600" windowHeight="11505" xr2:uid="{61C89FE4-8FBE-4549-A785-404B3EAD14AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Cloths" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="42">
   <si>
     <t>Elvs Braided curly beads hairdo</t>
   </si>
@@ -131,6 +131,27 @@
   </si>
   <si>
     <t>Gaunlet</t>
+  </si>
+  <si>
+    <t>Art And Logs</t>
+  </si>
+  <si>
+    <t>HoplesTheSnek</t>
+  </si>
+  <si>
+    <t>chinstrap</t>
+  </si>
+  <si>
+    <t>grinsegold</t>
+  </si>
+  <si>
+    <t>beard_and_mustache</t>
+  </si>
+  <si>
+    <t>Moustache</t>
+  </si>
+  <si>
+    <t>combover</t>
   </si>
 </sst>
 </file>
@@ -489,52 +510,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82F84505-55E1-44C9-8BC3-7EAD47638064}">
-  <dimension ref="A2:B23"/>
+  <dimension ref="A2:B28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
@@ -542,31 +563,31 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
@@ -574,7 +595,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
@@ -582,63 +603,63 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
         <v>28</v>
@@ -646,26 +667,66 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B23" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>